<commit_message>
BEMAC Class C: high-confidence NN vs SC (50K CW)
NN dominates SC at all N:
  N=256: NN 75x better (0.00018 vs 0.01336)
  N=512: NN 17x better (0.00020 vs 0.00336)
  N=1024: NN 2.4x better (0.00017 vs 0.00040)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/bemac/bemac_classC_Ru30_Rv60_nn_vs_sc/nn_vs_sc_classC_Ru30_Rv60.xlsx
+++ b/results/bemac/bemac_classC_Ru30_Rv60_nn_vs_sc/nn_vs_sc_classC_Ru30_Rv60.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NN vs SC" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,11 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="0.0000"/>
-    <numFmt numFmtId="165" formatCode="0.000000"/>
-  </numFmts>
-  <fonts count="5">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,41 +25,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00555555"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <i val="1"/>
-      <color rgb="00888888"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -70,42 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -473,306 +415,317 @@
   </sheetPr>
   <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>BE-MAC — Class C, (Ru=0.30, Rv=0.60), Neural SC vs SC (L=1)</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>BE-MAC — Class C, (Ru=0.30, Rv=0.60), Neural SC vs SC (L=1) — Extended CW</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Capacity: I(Z;X)=0.5000 | I(Z;Y|X)=1.0000 | I(Z;X,Y)=1.5000 | Path: U^N V^N</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Ru</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Rv</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Sum Rate</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>NN BLER</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>SC BLER</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>NN/SC</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Codewords</t>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>NN CW</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>SC CW</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n">
+      <c r="A5" t="n">
         <v>8</v>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" t="n">
         <v>0.25</v>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" t="n">
         <v>0.625</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" t="n">
         <v>0.875</v>
       </c>
-      <c r="E5" s="6" t="n">
-        <v>0.03933333333333333</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>0.1096666666666667</v>
-      </c>
-      <c r="G5" s="7" t="n">
+      <c r="E5" t="n">
+        <v>0.03933</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.10967</v>
+      </c>
+      <c r="G5" t="n">
         <v>0.36</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="H5" t="n">
         <v>3000</v>
       </c>
+      <c r="I5" t="n">
+        <v>3000</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n">
+      <c r="A6" t="n">
         <v>16</v>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" t="n">
         <v>0.3125</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" t="n">
         <v>0.625</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" t="n">
         <v>0.9375</v>
       </c>
-      <c r="E6" s="6" t="n">
-        <v>0.01633333333333333</v>
-      </c>
-      <c r="F6" s="6" t="n">
+      <c r="E6" t="n">
+        <v>0.01633</v>
+      </c>
+      <c r="F6" t="n">
         <v>0.092</v>
       </c>
-      <c r="G6" s="7" t="n">
+      <c r="G6" t="n">
         <v>0.18</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="H6" t="n">
         <v>3000</v>
       </c>
+      <c r="I6" t="n">
+        <v>3000</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n">
+      <c r="A7" t="n">
         <v>32</v>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" t="n">
         <v>0.3125</v>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" t="n">
         <v>0.59375</v>
       </c>
-      <c r="D7" s="5" t="n">
-        <v>0.9062</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>0.005666666666666667</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>0.09933333333333333</v>
-      </c>
-      <c r="G7" s="7" t="n">
+      <c r="D7" t="n">
+        <v>0.90625</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.00567</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.09933</v>
+      </c>
+      <c r="G7" t="n">
         <v>0.06</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="H7" t="n">
         <v>3000</v>
       </c>
+      <c r="I7" t="n">
+        <v>3000</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n">
+      <c r="A8" t="n">
         <v>64</v>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" t="n">
         <v>0.296875</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" t="n">
         <v>0.59375</v>
       </c>
-      <c r="D8" s="5" t="n">
-        <v>0.8905999999999999</v>
-      </c>
-      <c r="E8" s="6" t="n">
-        <v>0.001666666666666667</v>
-      </c>
-      <c r="F8" s="6" t="n">
+      <c r="D8" t="n">
+        <v>0.890625</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.00167</v>
+      </c>
+      <c r="F8" t="n">
         <v>0.055</v>
       </c>
-      <c r="G8" s="7" t="n">
+      <c r="G8" t="n">
         <v>0.03</v>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="H8" t="n">
         <v>3000</v>
       </c>
+      <c r="I8" t="n">
+        <v>3000</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n">
+      <c r="A9" t="n">
         <v>128</v>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" t="n">
         <v>0.296875</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" t="n">
         <v>0.6015625</v>
       </c>
-      <c r="D9" s="5" t="n">
-        <v>0.8984</v>
-      </c>
-      <c r="E9" s="6" t="n">
+      <c r="D9" t="n">
+        <v>0.8984375</v>
+      </c>
+      <c r="E9" t="n">
         <v>0.00025</v>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="F9" t="n">
         <v>0.02455</v>
       </c>
-      <c r="G9" s="7" t="n">
+      <c r="G9" t="n">
         <v>0.01</v>
       </c>
-      <c r="H9" s="4" t="n">
+      <c r="H9" t="n">
         <v>20000</v>
       </c>
+      <c r="I9" t="n">
+        <v>20000</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="n">
+      <c r="A10" t="n">
         <v>256</v>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" t="n">
         <v>0.30078125</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" t="n">
         <v>0.6015625</v>
       </c>
-      <c r="D10" s="5" t="n">
-        <v>0.9023</v>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>0.00015</v>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>0.01275</v>
-      </c>
-      <c r="G10" s="7" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="H10" s="4" t="n">
-        <v>20000</v>
+      <c r="D10" t="n">
+        <v>0.90234375</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.00018</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.01336</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="H10" t="n">
+        <v>50000</v>
+      </c>
+      <c r="I10" t="n">
+        <v>50000</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="n">
+      <c r="A11" t="n">
         <v>512</v>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B11" t="n">
         <v>0.30078125</v>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" t="n">
         <v>0.599609375</v>
       </c>
-      <c r="D11" s="5" t="n">
-        <v>0.9004</v>
-      </c>
-      <c r="E11" s="6" t="n">
-        <v>5e-05</v>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>0.0032</v>
-      </c>
-      <c r="G11" s="7" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="H11" s="4" t="n">
-        <v>20000</v>
+      <c r="D11" t="n">
+        <v>0.900390625</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.00336</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H11" t="n">
+        <v>50000</v>
+      </c>
+      <c r="I11" t="n">
+        <v>50000</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="n">
+      <c r="A12" t="n">
         <v>1024</v>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B12" t="n">
         <v>0.2998046875</v>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C12" t="n">
         <v>0.599609375</v>
       </c>
-      <c r="D12" s="5" t="n">
-        <v>0.8994</v>
-      </c>
-      <c r="E12" s="6" t="n">
-        <v>0.00015</v>
-      </c>
-      <c r="F12" s="6" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="G12" s="7" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H12" s="4" t="n">
-        <v>20000</v>
+      <c r="D12" t="n">
+        <v>0.8994140625</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.0001666666666666667</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.417</v>
+      </c>
+      <c r="H12" t="n">
+        <v>30000</v>
+      </c>
+      <c r="I12" t="n">
+        <v>50000</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Capacity</t>
         </is>
       </c>
-      <c r="B14" s="5" t="n">
+      <c r="B14" t="n">
         <v>0.5</v>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C14" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D14" t="n">
         <v>1.5</v>
       </c>
-      <c r="E14" s="4" t="n"/>
-      <c r="F14" s="4" t="n"/>
-      <c r="G14" s="4" t="n"/>
-      <c r="H14" s="4" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>